<commit_message>
#110 eSpark And JLCPCB BOM and Deliverables Updated
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Electrode-Board/JLCPCB-BOM -Elect-Board.xlsx
+++ b/Deliverables/BOM/Electrode-Board/JLCPCB-BOM -Elect-Board.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ManarHarake-sEMGDevice\Deliverables\BOM\Electrode-Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8044EFD-544D-4A4E-98BC-565A4CB9877F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F892935-E1EE-409B-BCAD-549B91666FE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="120" yWindow="-120" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="52">
   <si>
     <t>Comment</t>
   </si>
@@ -64,18 +64,12 @@
     <t>Designator</t>
   </si>
   <si>
-    <t>C1, C5</t>
-  </si>
-  <si>
     <t>C2, C6</t>
   </si>
   <si>
     <t>C3</t>
   </si>
   <si>
-    <t>C4</t>
-  </si>
-  <si>
     <t>D1, D2</t>
   </si>
   <si>
@@ -109,9 +103,6 @@
     <t>Footprint</t>
   </si>
   <si>
-    <t>Cap-0603</t>
-  </si>
-  <si>
     <t>Cap-0402</t>
   </si>
   <si>
@@ -142,9 +133,6 @@
     <t>LCSC Part Number</t>
   </si>
   <si>
-    <t>C106214</t>
-  </si>
-  <si>
     <t>C182412</t>
   </si>
   <si>
@@ -185,6 +173,9 @@
   </si>
   <si>
     <t>C514366</t>
+  </si>
+  <si>
+    <t>C1, C4, C5</t>
   </si>
 </sst>
 </file>
@@ -658,7 +649,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -675,10 +666,10 @@
         <v>13</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -686,13 +677,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -700,13 +691,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -714,167 +705,153 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D7" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="6" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="5" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="D12" s="6" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D14" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>54</v>
+      <c r="B14" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>